<commit_message>
fix: critical correctness bugs (timezone, source-leak, unknown-column)
- Date canonical string is UTC-based per ADR-0017, was reading local
  timezone components (off-by-one day in any non-UTC host).
- `__sources__[Name]` reserved-ref form now errors with
  xl3/sources/not-a-dictionary instead of leaking the internal source
  descriptor.
- Source[Column] referencing an undeclared column errors with
  xl3/source/unknown-column instead of silently aggregating to 0; the
  same check covers XLOOKUP arg 2/3 and bare [Column] in @source blocks.
- Aux-sheet cleanup matches the dunder-wrapped reserved sheet form per
  ADR-0011 (was matching legacy `_`-prefix only).
- Date inputs, Excel-serial conversion, and strict date parsing all
  build via Date.UTC for round-trip stability.

Conformance: 87/91 pass (4 stage-2 skipped). Fixture 091 added for the
unknown-column error. Fixtures 009/011/087/088 rebuilt with UTC-anchored
dates so the canonical-string contract holds on any host timezone.
</commit_message>
<xml_diff>
--- a/conformance/fixtures/087-date-canonical-string-concat/data.xlsx
+++ b/conformance/fixtures/087-date-canonical-string-concat/data.xlsx
@@ -421,7 +421,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="1">
-        <v>46149.625</v>
+        <v>46150</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -429,7 +429,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="2">
-        <v>46150.02083333333</v>
+        <v>46150.39583333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>